<commit_message>
Updated Answer keys fpr HRM, MM, OM, FM
</commit_message>
<xml_diff>
--- a/Data/FM/FM_Quizzes.xlsx
+++ b/Data/FM/FM_Quizzes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\mba_quiz\Data\FM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0C7CAA-8443-4333-805B-0419CC9908B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F44100-A837-417B-AC68-3D9907134093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="757" xr2:uid="{850D3C83-EED4-4016-BDB5-EF8EECDCB418}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="757" firstSheet="1" activeTab="11" xr2:uid="{850D3C83-EED4-4016-BDB5-EF8EECDCB418}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="26" r:id="rId1"/>
@@ -4088,7 +4088,7 @@
         <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4134,7 +4134,7 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4180,7 +4180,7 @@
         <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -4203,7 +4203,7 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -4272,7 +4272,7 @@
         <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -4295,7 +4295,7 @@
         <v>54</v>
       </c>
       <c r="G11" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -4318,7 +4318,7 @@
         <v>60</v>
       </c>
       <c r="G12" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -4341,7 +4341,7 @@
         <v>66</v>
       </c>
       <c r="G13" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -4364,7 +4364,7 @@
         <v>72</v>
       </c>
       <c r="G14" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -4387,7 +4387,7 @@
         <v>77</v>
       </c>
       <c r="G15" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>83</v>
       </c>
       <c r="G16" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -4433,7 +4433,7 @@
         <v>89</v>
       </c>
       <c r="G17" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -4456,7 +4456,7 @@
         <v>95</v>
       </c>
       <c r="G18" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -4502,7 +4502,7 @@
         <v>104</v>
       </c>
       <c r="G20" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -4525,7 +4525,7 @@
         <v>109</v>
       </c>
       <c r="G21" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
   </sheetData>
@@ -4593,7 +4593,7 @@
         <v>795</v>
       </c>
       <c r="G2" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4616,7 +4616,7 @@
         <v>800</v>
       </c>
       <c r="G3" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -4639,7 +4639,7 @@
         <v>805</v>
       </c>
       <c r="G4" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4662,7 +4662,7 @@
         <v>807</v>
       </c>
       <c r="G5" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -4685,7 +4685,7 @@
         <v>812</v>
       </c>
       <c r="G6" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -4708,7 +4708,7 @@
         <v>333</v>
       </c>
       <c r="G7" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -4731,7 +4731,7 @@
         <v>816</v>
       </c>
       <c r="G8" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -4777,7 +4777,7 @@
         <v>283</v>
       </c>
       <c r="G10" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -4800,7 +4800,7 @@
         <v>598</v>
       </c>
       <c r="G11" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -4823,7 +4823,7 @@
         <v>830</v>
       </c>
       <c r="G12" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -4869,7 +4869,7 @@
         <v>612</v>
       </c>
       <c r="G14" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -4892,7 +4892,7 @@
         <v>838</v>
       </c>
       <c r="G15" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -4915,7 +4915,7 @@
         <v>843</v>
       </c>
       <c r="G16" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -4938,7 +4938,7 @@
         <v>847</v>
       </c>
       <c r="G17" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>852</v>
       </c>
       <c r="G18" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -4984,7 +4984,7 @@
         <v>855</v>
       </c>
       <c r="G19" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -5007,7 +5007,7 @@
         <v>407</v>
       </c>
       <c r="G20" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -5030,7 +5030,7 @@
         <v>863</v>
       </c>
       <c r="G21" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
   </sheetData>
@@ -5306,7 +5306,7 @@
         <v>900</v>
       </c>
       <c r="G11" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -5604,7 +5604,7 @@
         <v>943</v>
       </c>
       <c r="G2" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -6110,7 +6110,7 @@
         <v>114</v>
       </c>
       <c r="G2" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -6133,7 +6133,7 @@
         <v>119</v>
       </c>
       <c r="G3" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>129</v>
       </c>
       <c r="G5" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -6202,7 +6202,7 @@
         <v>134</v>
       </c>
       <c r="G6" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -6225,7 +6225,7 @@
         <v>139</v>
       </c>
       <c r="G7" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -6248,7 +6248,7 @@
         <v>134</v>
       </c>
       <c r="G8" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -6271,7 +6271,7 @@
         <v>148</v>
       </c>
       <c r="G9" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -6317,7 +6317,7 @@
         <v>158</v>
       </c>
       <c r="G11" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -6340,7 +6340,7 @@
         <v>163</v>
       </c>
       <c r="G12" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -6386,7 +6386,7 @@
         <v>1034</v>
       </c>
       <c r="G14" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -6409,7 +6409,7 @@
         <v>174</v>
       </c>
       <c r="G15" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -6432,7 +6432,7 @@
         <v>179</v>
       </c>
       <c r="G16" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -6455,7 +6455,7 @@
         <v>184</v>
       </c>
       <c r="G17" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -6501,7 +6501,7 @@
         <v>194</v>
       </c>
       <c r="G19" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -6547,7 +6547,7 @@
         <v>204</v>
       </c>
       <c r="G21" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
   </sheetData>
@@ -6615,7 +6615,7 @@
         <v>209</v>
       </c>
       <c r="G2" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -6638,7 +6638,7 @@
         <v>214</v>
       </c>
       <c r="G3" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -6661,7 +6661,7 @@
         <v>219</v>
       </c>
       <c r="G4" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6684,7 +6684,7 @@
         <v>224</v>
       </c>
       <c r="G5" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -6707,7 +6707,7 @@
         <v>229</v>
       </c>
       <c r="G6" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>234</v>
       </c>
       <c r="G7" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -6776,7 +6776,7 @@
         <v>217</v>
       </c>
       <c r="G9" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -6799,7 +6799,7 @@
         <v>247</v>
       </c>
       <c r="G10" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -6845,7 +6845,7 @@
         <v>257</v>
       </c>
       <c r="G12" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -6891,7 +6891,7 @@
         <v>266</v>
       </c>
       <c r="G14" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -6914,7 +6914,7 @@
         <v>271</v>
       </c>
       <c r="G15" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -6937,7 +6937,7 @@
         <v>251</v>
       </c>
       <c r="G16" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -7006,7 +7006,7 @@
         <v>289</v>
       </c>
       <c r="G19" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -7029,7 +7029,7 @@
         <v>121</v>
       </c>
       <c r="G20" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -7052,7 +7052,7 @@
         <v>296</v>
       </c>
       <c r="G21" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
   </sheetData>
@@ -7120,7 +7120,7 @@
         <v>300</v>
       </c>
       <c r="G2" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -7143,7 +7143,7 @@
         <v>305</v>
       </c>
       <c r="G3" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -7166,7 +7166,7 @@
         <v>310</v>
       </c>
       <c r="G4" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -7189,7 +7189,7 @@
         <v>315</v>
       </c>
       <c r="G5" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -7212,7 +7212,7 @@
         <v>320</v>
       </c>
       <c r="G6" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -7235,7 +7235,7 @@
         <v>131</v>
       </c>
       <c r="G7" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -7258,7 +7258,7 @@
         <v>313</v>
       </c>
       <c r="G8" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>122</v>
       </c>
       <c r="G9" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -7304,7 +7304,7 @@
         <v>333</v>
       </c>
       <c r="G10" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -7327,7 +7327,7 @@
         <v>338</v>
       </c>
       <c r="G11" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -7350,7 +7350,7 @@
         <v>343</v>
       </c>
       <c r="G12" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -7396,7 +7396,7 @@
         <v>352</v>
       </c>
       <c r="G14" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -7419,7 +7419,7 @@
         <v>357</v>
       </c>
       <c r="G15" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -7442,7 +7442,7 @@
         <v>362</v>
       </c>
       <c r="G16" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -7465,7 +7465,7 @@
         <v>367</v>
       </c>
       <c r="G17" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -7488,7 +7488,7 @@
         <v>370</v>
       </c>
       <c r="G18" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -7511,7 +7511,7 @@
         <v>375</v>
       </c>
       <c r="G19" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -7534,7 +7534,7 @@
         <v>380</v>
       </c>
       <c r="G20" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -7557,7 +7557,7 @@
         <v>283</v>
       </c>
       <c r="G21" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
   </sheetData>
@@ -7648,7 +7648,7 @@
         <v>392</v>
       </c>
       <c r="G3" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -7671,7 +7671,7 @@
         <v>397</v>
       </c>
       <c r="G4" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -7694,7 +7694,7 @@
         <v>402</v>
       </c>
       <c r="G5" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -7740,7 +7740,7 @@
         <v>409</v>
       </c>
       <c r="G7" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -7763,7 +7763,7 @@
         <v>414</v>
       </c>
       <c r="G8" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -7786,7 +7786,7 @@
         <v>418</v>
       </c>
       <c r="G9" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>426</v>
       </c>
       <c r="G11" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -7855,7 +7855,7 @@
         <v>390</v>
       </c>
       <c r="G12" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -7878,7 +7878,7 @@
         <v>178</v>
       </c>
       <c r="G13" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -7901,7 +7901,7 @@
         <v>436</v>
       </c>
       <c r="G14" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -7924,7 +7924,7 @@
         <v>407</v>
       </c>
       <c r="G15" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -7947,7 +7947,7 @@
         <v>444</v>
       </c>
       <c r="G16" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -7970,7 +7970,7 @@
         <v>447</v>
       </c>
       <c r="G17" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -8016,7 +8016,7 @@
         <v>456</v>
       </c>
       <c r="G19" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -8039,7 +8039,7 @@
         <v>461</v>
       </c>
       <c r="G20" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -8062,7 +8062,7 @@
         <v>466</v>
       </c>
       <c r="G21" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
   </sheetData>
@@ -8130,7 +8130,7 @@
         <v>470</v>
       </c>
       <c r="G2" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -8153,7 +8153,7 @@
         <v>473</v>
       </c>
       <c r="G3" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -8176,7 +8176,7 @@
         <v>477</v>
       </c>
       <c r="G4" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -8199,7 +8199,7 @@
         <v>482</v>
       </c>
       <c r="G5" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -8222,7 +8222,7 @@
         <v>487</v>
       </c>
       <c r="G6" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -8245,7 +8245,7 @@
         <v>492</v>
       </c>
       <c r="G7" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -8291,7 +8291,7 @@
         <v>501</v>
       </c>
       <c r="G9" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -8429,7 +8429,7 @@
         <v>524</v>
       </c>
       <c r="G15" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -8452,7 +8452,7 @@
         <v>123</v>
       </c>
       <c r="G16" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -8475,7 +8475,7 @@
         <v>529</v>
       </c>
       <c r="G17" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -8521,7 +8521,7 @@
         <v>407</v>
       </c>
       <c r="G19" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -8567,7 +8567,7 @@
         <v>547</v>
       </c>
       <c r="G21" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
   </sheetData>
@@ -8635,7 +8635,7 @@
         <v>552</v>
       </c>
       <c r="G2" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -8658,7 +8658,7 @@
         <v>557</v>
       </c>
       <c r="G3" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -8681,7 +8681,7 @@
         <v>562</v>
       </c>
       <c r="G4" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -8704,7 +8704,7 @@
         <v>567</v>
       </c>
       <c r="G5" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -8727,7 +8727,7 @@
         <v>572</v>
       </c>
       <c r="G6" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -8750,7 +8750,7 @@
         <v>575</v>
       </c>
       <c r="G7" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -8796,7 +8796,7 @@
         <v>585</v>
       </c>
       <c r="G9" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -8819,7 +8819,7 @@
         <v>590</v>
       </c>
       <c r="G10" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -8842,7 +8842,7 @@
         <v>594</v>
       </c>
       <c r="G11" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -8865,7 +8865,7 @@
         <v>599</v>
       </c>
       <c r="G12" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -8888,7 +8888,7 @@
         <v>604</v>
       </c>
       <c r="G13" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -8911,7 +8911,7 @@
         <v>609</v>
       </c>
       <c r="G14" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -9003,7 +9003,7 @@
         <v>628</v>
       </c>
       <c r="G18" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -9072,7 +9072,7 @@
         <v>641</v>
       </c>
       <c r="G21" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
   </sheetData>
@@ -9140,7 +9140,7 @@
         <v>719</v>
       </c>
       <c r="G2" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -9163,7 +9163,7 @@
         <v>724</v>
       </c>
       <c r="G3" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -9186,7 +9186,7 @@
         <v>729</v>
       </c>
       <c r="G4" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -9209,7 +9209,7 @@
         <v>734</v>
       </c>
       <c r="G5" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -9232,7 +9232,7 @@
         <v>192</v>
       </c>
       <c r="G6" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -9255,7 +9255,7 @@
         <v>741</v>
       </c>
       <c r="G7" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -9278,7 +9278,7 @@
         <v>447</v>
       </c>
       <c r="G8" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -9301,7 +9301,7 @@
         <v>611</v>
       </c>
       <c r="G9" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -9324,7 +9324,7 @@
         <v>733</v>
       </c>
       <c r="G10" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -9370,7 +9370,7 @@
         <v>758</v>
       </c>
       <c r="G12" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -9393,7 +9393,7 @@
         <v>407</v>
       </c>
       <c r="G13" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -9416,7 +9416,7 @@
         <v>1030</v>
       </c>
       <c r="G14" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -9439,7 +9439,7 @@
         <v>767</v>
       </c>
       <c r="G15" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -9462,7 +9462,7 @@
         <v>772</v>
       </c>
       <c r="G16" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -9508,7 +9508,7 @@
         <v>777</v>
       </c>
       <c r="G18" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -9531,7 +9531,7 @@
         <v>782</v>
       </c>
       <c r="G19" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -9554,7 +9554,7 @@
         <v>786</v>
       </c>
       <c r="G20" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -9668,7 +9668,7 @@
         <v>650</v>
       </c>
       <c r="G3" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -9691,7 +9691,7 @@
         <v>655</v>
       </c>
       <c r="G4" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -9714,7 +9714,7 @@
         <v>439</v>
       </c>
       <c r="G5" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -9737,7 +9737,7 @@
         <v>664</v>
       </c>
       <c r="G6" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -9760,7 +9760,7 @@
         <v>669</v>
       </c>
       <c r="G7" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -9806,7 +9806,7 @@
         <v>677</v>
       </c>
       <c r="G9" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -9829,7 +9829,7 @@
         <v>193</v>
       </c>
       <c r="G10" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -9875,7 +9875,7 @@
         <v>685</v>
       </c>
       <c r="G12" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -9898,7 +9898,7 @@
         <v>71</v>
       </c>
       <c r="G13" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -9990,7 +9990,7 @@
         <v>598</v>
       </c>
       <c r="G17" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -10013,7 +10013,7 @@
         <v>705</v>
       </c>
       <c r="G18" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>709</v>
       </c>
       <c r="G19" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -10082,7 +10082,7 @@
         <v>717</v>
       </c>
       <c r="G21" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
   </sheetData>

</xml_diff>